<commit_message>
Point the upstream sync procedure at version-6.2-main.
The Oct 14 sync now lives on that branch, so the next integration branch is cut from there.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/upstream/manual-regression-checklist-qa.xlsx
+++ b/docs/upstream/manual-regression-checklist-qa.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Checklist" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Run info" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Dedup log" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run info" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dedup log" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist'!$A$1:$I$138</definedName>
@@ -570,7 +570,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>1. On version-6.1-main: bun run apps/sim/scripts/diff-block-output-contracts.ts dump --out /tmp/output-contracts-before.json
+          <t>1. On version-6.2-main: bun run apps/sim/scripts/diff-block-output-contracts.ts dump --out /tmp/output-contracts-before.json
 2. On the sync branch: bun run apps/sim/scripts/diff-block-output-contracts.ts diff /tmp/output-contracts-before.json
 3. Compare removals/type changes to the sync report.</t>
         </is>

</xml_diff>

<commit_message>
sugestion follow up updtated regression
</commit_message>
<xml_diff>
--- a/docs/upstream/manual-regression-checklist-qa.xlsx
+++ b/docs/upstream/manual-regression-checklist-qa.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dedup log" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist'!$A$1:$I$138</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist'!$A$1:$I$139</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Dedup log'!$A$1:$C$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I138"/>
+  <dimension ref="A1:I139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1795,18 +1795,20 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Finished Copilot reply does not turn asterisks into bold on scroll</t>
+          <t>Local fork still opens a new chat when the worker has no conversation</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>1. Get a Copilot reply that contains ordinary * characters or unfinished markdown.
-2. Wait until the reply has finished, then scroll the thread away and back.</t>
+          <t>1. On Local, finish at least one Copilot reply.
+2. Use Fork in new chat on that reply.
+3. Confirm the new chat opens with a title starting Fork | and the messages up to that reply.
+4. On Cloud, with COPILOT_API_KEY set, fork a finished reply the same way.</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>The finished text stays as it streamed. Scrolling does not turn those characters into bold.</t>
+          <t>Local fork opens the new chat. There is no “Failed to fork chat” toast. Cloud fork still succeeds and keeps the worker conversation.</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr"/>
@@ -1828,62 +1830,62 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Finished Copilot reply does not turn asterisks into bold on scroll</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>1. Get a Copilot reply that contains ordinary * characters or unfinished markdown.
+2. Wait until the reply has finished, then scroll the thread away and back.</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>The finished text stays as it streamed. Scrolling does not turn those characters into bold.</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="90" customHeight="1">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>1. Customized — Sim behavior Arena changed</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Workspace chat and Local/Cloud copilot</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>Fetch-and-send sequence is canvas blocks, not Agent tools</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>1. Ask Copilot: today’s calendar, unread Gmail, Slack messages, then a written briefing.
 2. Also ask for a daily time trigger.
 3. Inspect the canvas block types and the Agent tools list.</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>The canvas has google_calendar_v2, gmail_v2, and slack as their own blocks in that order. Those integrations are not Agent tools. The daily trigger is a schedule block, not schedule_trigger.</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr"/>
-      <c r="I36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37" ht="90" customHeight="1">
-      <c r="A37" s="2" t="n">
-        <v>36</v>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>1. Customized — Sim behavior Arena changed</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>Workspace chat and Local/Cloud copilot</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>Copilot HTML file opens as a complete page</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>1. Ask Copilot to create an HTML page.
-2. Open the saved file.</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t>The file opens as a complete page. The chat does not dump a truncated tag soup in place of the file.</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr"/>
@@ -1905,62 +1907,62 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
+          <t>Copilot HTML file opens as a complete page</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>1. Ask Copilot to create an HTML page.
+2. Open the saved file.</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>The file opens as a complete page. The chat does not dump a truncated tag soup in place of the file.</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="90" customHeight="1">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>1. Customized — Sim behavior Arena changed</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Workspace chat and Local/Cloud copilot</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
           <t>Local-only users stay on Local without the switch</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>1. Sign in as a localOnly allowlisted user.
 2. Open home and workflow Copilot.
 3. Send a message (even if a stale Cloud preference exists).</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>No Local/Cloud switch. Sends stay on Local.</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr"/>
-      <c r="I38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39" ht="90" customHeight="1">
-      <c r="A39" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>1. Customized — Sim behavior Arena changed</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>Workspace chat and Local/Cloud copilot</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>Copilot images/files land on Arena ledger</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t>1. From Copilot, generate an image and create a file on Local.
-2. Open Usage / ledger.</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>Image/file usage appears on the Arena ledger for the Local turns.</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
@@ -1987,18 +1989,18 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Floating workflow chat streams chart/image</t>
+          <t>Copilot images/files land on Arena ledger</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>1. Open floating workflow chat.
-2. Run a prompt that produces chart and/or image output.</t>
+          <t>1. From Copilot, generate an image and create a file on Local.
+2. Open Usage / ledger.</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Run streams; chart and image output render in the floating chat.</t>
+          <t>Image/file usage appears on the Arena ledger for the Local turns.</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
@@ -2025,18 +2027,18 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Deploy-modal chat preview matches deployed agent</t>
+          <t>Floating workflow chat streams chart/image</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>1. Open deploy modal chat preview for an agent.
-2. Compare theming/welcome behaviour to the live deployed URL.</t>
+          <t>1. Open floating workflow chat.
+2. Run a prompt that produces chart and/or image output.</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Preview matches the deployed agent experience (theme, welcome, basic send).</t>
+          <t>Run streams; chart and image output render in the floating chat.</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
@@ -2053,67 +2055,67 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
+          <t>Workspace chat and Local/Cloud copilot</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Deploy-modal chat preview matches deployed agent</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>1. Open deploy modal chat preview for an agent.
+2. Compare theming/welcome behaviour to the live deployed URL.</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Preview matches the deployed agent experience (theme, welcome, basic send).</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="90" customHeight="1">
+      <c r="A43" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>1. Customized — Sim behavior Arena changed</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
           <t>Billing and workspaces</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
         <is>
           <t>Credits debit matches ledger after one Agent turn</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F43" s="2" t="inlineStr">
         <is>
           <t>1. Note remaining credits / known balance.
 2. Run one Agent turn.
 3. Compare Usage dashboard debit to the ledger entry (credits-per-dollar).</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G43" s="2" t="inlineStr">
         <is>
           <t>Dashboard debit matches the ledger entry for that turn. No unexplained extra debit.</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr"/>
-      <c r="I42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43" ht="90" customHeight="1">
-      <c r="A43" s="2" t="n">
-        <v>42</v>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>1. Customized — Sim behavior Arena changed</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>Billing and workspaces</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>Cost block amount shows once (no double charge)</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>1. Run a workflow with an Agent model cost and an explicit Cost block amount.
-2. Inspect the run’s usage rows.</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>Explicit Cost block amount appears once. No double charge vs the Agent model cost.</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -2140,18 +2142,18 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Usage-log multiplier: one scaled ledger row</t>
+          <t>Cost block amount shows once (no double charge)</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>1. Run a metered tool that uses the usage-log multiplier.
-2. Inspect ledger rows for that run.</t>
+          <t>1. Run a workflow with an Agent model cost and an explicit Cost block amount.
+2. Inspect the run’s usage rows.</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Exactly one scaled ledger row is written — not a raw row plus a scaled duplicate.</t>
+          <t>Explicit Cost block amount appears once. No double charge vs the Agent model cost.</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
@@ -2178,18 +2180,18 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Signup personal workspace; /workspace fallback</t>
+          <t>Usage-log multiplier: one scaled ledger row</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>1. Sign up a new user (or use a fresh account path).
-2. Visit /workspace with no id.</t>
+          <t>1. Run a metered tool that uses the usage-log multiplier.
+2. Inspect ledger rows for that run.</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Signup creates a personal workspace. /workspace fallback lands on a valid workspace.</t>
+          <t>Exactly one scaled ledger row is written — not a raw row plus a scaled duplicate.</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr"/>
@@ -2216,49 +2218,87 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
+          <t>Signup personal workspace; /workspace fallback</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>1. Sign up a new user (or use a fresh account path).
+2. Visit /workspace with no id.</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Signup creates a personal workspace. /workspace fallback lands on a valid workspace.</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr"/>
+      <c r="I46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47" ht="90" customHeight="1">
+      <c r="A47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>1. Customized — Sim behavior Arena changed</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Billing and workspaces</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
           <t>Daily credit refresh off unless explicitly enabled</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>1. Confirm env does not enable daily refresh (default Arena).
 2. Observe that daily refresh does not run.
 3. If a test env enables it, confirm it then runs.</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t>Daily refresh stays off by default. It only runs when the environment explicitly enables it.</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr"/>
-      <c r="I46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47" ht="90" customHeight="1">
-      <c r="A47" s="2" t="n">
-        <v>46</v>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="H47" s="2" t="inlineStr"/>
+      <c r="I47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48" ht="90" customHeight="1">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>1. Customized — Sim behavior Arena changed</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>Billing and workspaces</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>X-Sim-Email bills the named user’s org once</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>1. Open the deploy-modal API sample and confirm X-Sim-Email is present.
 2. Execute the workflow API with X-Sim-Email set to a Sim user in another organization.
@@ -2266,47 +2306,9 @@
 4. Repeat with a missing header, a malformed email, and an email that matches no user.</t>
         </is>
       </c>
-      <c r="G47" s="2" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>The run bills the named user’s org once. The owning workspace does not also debit it. The billed org’s Usage shows a By Agent row (workflow, owning org · workspace, Run by) and remaining credits drop by that run. A missing header or malformed email is 400. An unknown email is 400 with BILLING_EMAIL_NOT_FOUND.</t>
-        </is>
-      </c>
-      <c r="H47" s="2" t="inlineStr"/>
-      <c r="I47" s="2" t="inlineStr"/>
-    </row>
-    <row r="48" ht="90" customHeight="1">
-      <c r="A48" s="2" t="n">
-        <v>47</v>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>1. Customized — Sim behavior Arena changed</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Workflow engine</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>Response inside loop continues; outside ends</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>1. Build a loop with a Response inside; run.
-2. Build a workflow with a Response outside any loop; run.</t>
-        </is>
-      </c>
-      <c r="G48" s="2" t="inlineStr">
-        <is>
-          <t>Response inside a loop continues the loop. Response outside a loop ends the workflow.</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -2333,18 +2335,18 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Empty forEach still runs the block after the loop</t>
+          <t>Response inside loop continues; outside ends</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>1. Build a forEach over an empty collection with a successor block after the loop.
-2. Run the workflow.</t>
+          <t>1. Build a loop with a Response inside; run.
+2. Build a workflow with a Response outside any loop; run.</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Loop body is skipped. The block after the loop still executes.</t>
+          <t>Response inside a loop continues the loop. Response outside a loop ends the workflow.</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -2371,18 +2373,18 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Nested loops and nested subflows save and run</t>
+          <t>Empty forEach still runs the block after the loop</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>1. Create nested loops / nested subflows (Arena allows; upstream rejects).
-2. Save and run.</t>
+          <t>1. Build a forEach over an empty collection with a successor block after the loop.
+2. Run the workflow.</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Nested structures save and run successfully.</t>
+          <t>Loop body is skipped. The block after the loop still executes.</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -2409,57 +2411,57 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
+          <t>Nested loops and nested subflows save and run</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>1. Create nested loops / nested subflows (Arena allows; upstream rejects).
+2. Save and run.</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Nested structures save and run successfully.</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr"/>
+      <c r="I51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52" ht="90" customHeight="1">
+      <c r="A52" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>1. Customized — Sim behavior Arena changed</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Workflow engine</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
           <t>Agent model picker: OpenRouter free-only; Azure Anthropic + image models</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>1. Open Agent model picker.
 2. Inspect OpenRouter list pricing.
 3. Confirm Azure Anthropic and Arena-added image models appear where expected.</t>
         </is>
       </c>
-      <c r="G51" s="2" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>OpenRouter list is free-only. Azure Anthropic and Arena image models still appear.</t>
-        </is>
-      </c>
-      <c r="H51" s="2" t="inlineStr"/>
-      <c r="I51" s="2" t="inlineStr"/>
-    </row>
-    <row r="52" ht="90" customHeight="1">
-      <c r="A52" s="2" t="n">
-        <v>51</v>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>1. Customized — Sim behavior Arena changed</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>Workflow engine</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>Run logs/console show charts, images, acting user</t>
-        </is>
-      </c>
-      <c r="F52" s="2" t="inlineStr">
-        <is>
-          <t>1. Run a workflow that produces chart and image payloads.
-2. Open console and logs for the run.</t>
-        </is>
-      </c>
-      <c r="G52" s="2" t="inlineStr">
-        <is>
-          <t>Chart payloads, image payloads, and the acting user are visible in run logs/console.</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
@@ -2476,106 +2478,106 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
+          <t>Workflow engine</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Run logs/console show charts, images, acting user</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>1. Run a workflow that produces chart and image payloads.
+2. Open console and logs for the run.</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Chart payloads, image payloads, and the acting user are visible in run logs/console.</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr"/>
+      <c r="I53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54" ht="90" customHeight="1">
+      <c r="A54" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>1. Customized — Sim behavior Arena changed</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
           <t>Extended integrations</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>Slack: Arena Bot and Custom Bot, search, post, and Copilot Connect</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>1. In the Slack block, select Arena Bot (bot token) and Custom Bot (user token).
 2. Run Slack search, user-channel lookup, and a normal post.
 3. Ask Copilot to connect Slack while it is disconnected.</t>
         </is>
       </c>
-      <c r="G53" s="2" t="inlineStr">
+      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>Both auth methods are selectable. Search, lookup, and post each succeed once. Copilot shows one Connect control (“Connect these, then continue”, button Continue), not a Submit button and not a repeated card.</t>
         </is>
       </c>
-      <c r="H53" s="2" t="inlineStr"/>
-      <c r="I53" s="2" t="inlineStr"/>
-    </row>
-    <row r="54" ht="90" customHeight="1">
-      <c r="A54" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="H54" s="2" t="inlineStr"/>
+      <c r="I54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55" ht="90" customHeight="1">
+      <c r="A55" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
         <is>
           <t>1. Customized — Sim behavior Arena changed</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
+      <c r="C55" s="2" t="inlineStr">
         <is>
           <t>Extended integrations</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="D55" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="E55" s="2" t="inlineStr">
         <is>
           <t>HubSpot: Accounts picker, campaign op, list contacts</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F55" s="2" t="inlineStr">
         <is>
           <t>1. On an admin workspace, open the HubSpot block and load the Accounts picker.
 2. Select an account and run a read.
 3. Run hubspot_get_campaign_metrics (or another campaign op) and stock hubspot_list_contacts.</t>
         </is>
       </c>
-      <c r="G54" s="2" t="inlineStr">
+      <c r="G55" s="2" t="inlineStr">
         <is>
           <t>The picker loads real portals and the selected account reads successfully. Campaign op and list contacts both return data.</t>
-        </is>
-      </c>
-      <c r="H54" s="2" t="inlineStr"/>
-      <c r="I54" s="2" t="inlineStr"/>
-    </row>
-    <row r="55" ht="90" customHeight="1">
-      <c r="A55" s="2" t="n">
-        <v>54</v>
-      </c>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>1. Customized — Sim behavior Arena changed</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>Extended integrations</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>Google Slides: template tables + stock slide action</t>
-        </is>
-      </c>
-      <c r="F55" s="2" t="inlineStr">
-        <is>
-          <t>1. Run create-from-template / template tables (Arena path).
-2. Run one stock slide action.</t>
-        </is>
-      </c>
-      <c r="G55" s="2" t="inlineStr">
-        <is>
-          <t>Template tables path and stock slide action each succeed once.</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -2602,18 +2604,18 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Zoom: recordings, transcript download, stock meeting</t>
+          <t>Google Slides: template tables + stock slide action</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>1. Fetch account recordings and download a transcript.
-2. Run one stock meeting action.</t>
+          <t>1. Run create-from-template / template tables (Arena path).
+2. Run one stock slide action.</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Recordings/transcript path and stock meeting action succeed.</t>
+          <t>Template tables path and stock slide action each succeed once.</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -2640,57 +2642,57 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
+          <t>Zoom: recordings, transcript download, stock meeting</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>1. Fetch account recordings and download a transcript.
+2. Run one stock meeting action.</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Recordings/transcript path and stock meeting action succeed.</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr"/>
+      <c r="I57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58" ht="90" customHeight="1">
+      <c r="A58" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>1. Customized — Sim behavior Arena changed</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Extended integrations</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
           <t>Shopify list customers (success) + list products</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr">
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>1. Run shopify_list_customers; assert downstream can read success.
 2. Run stock shopify_list_products.
 3. Optionally list/get another resource that previously mapped outputs.</t>
         </is>
       </c>
-      <c r="G57" s="2" t="inlineStr">
+      <c r="G58" s="2" t="inlineStr">
         <is>
           <t>list_customers succeeds and success remains available downstream. list_products succeeds. Output mapping intact.</t>
-        </is>
-      </c>
-      <c r="H57" s="2" t="inlineStr"/>
-      <c r="I57" s="2" t="inlineStr"/>
-    </row>
-    <row r="58" ht="90" customHeight="1">
-      <c r="A58" s="2" t="n">
-        <v>57</v>
-      </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>1. Customized — Sim behavior Arena changed</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>Extended integrations</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>Gmail: advanced search, read thread, send/read</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>1. Run advanced search and read thread.
-2. Send or read a message.</t>
-        </is>
-      </c>
-      <c r="G58" s="2" t="inlineStr">
-        <is>
-          <t>Advanced search/thread and send/read each succeed once.</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -2717,18 +2719,18 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Google Drive: upload, AI query helpers, stock file read</t>
+          <t>Gmail: advanced search, read thread, send/read</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>1. Upload a file and run an AI query helper.
-2. Run a stock file read / search.</t>
+          <t>1. Run advanced search and read thread.
+2. Send or read a message.</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Upload, AI query helpers, and stock file read/search succeed.</t>
+          <t>Advanced search/thread and send/read each succeed once.</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
@@ -2755,18 +2757,18 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Google Ads v26 search: results consumed as array</t>
+          <t>Google Drive: upload, AI query helpers, stock file read</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>1. Run Google Ads search (GAQL) and confirm the request uses API v26.
-2. Wire a downstream block to results (e.g. forEach or Function).</t>
+          <t>1. Upload a file and run an AI query helper.
+2. Run a stock file read / search.</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Search succeeds on v26. Downstream consumes results as an array (not a bare object / undefined).</t>
+          <t>Upload, AI query helpers, and stock file read/search succeed.</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr"/>
@@ -2793,96 +2795,96 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
+          <t>Google Ads v26 search: results consumed as array</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>1. Run Google Ads search (GAQL) and confirm the request uses API v26.
+2. Wire a downstream block to results (e.g. forEach or Function).</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Search succeeds on v26. Downstream consumes results as an array (not a bare object / undefined).</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr"/>
+      <c r="I61" s="2" t="inlineStr"/>
+    </row>
+    <row r="62" ht="90" customHeight="1">
+      <c r="A62" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>1. Customized — Sim behavior Arena changed</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Extended integrations</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
           <t>Image Generator: distinct variations, refs, edit</t>
         </is>
       </c>
-      <c r="F61" s="2" t="inlineStr">
+      <c r="F62" s="2" t="inlineStr">
         <is>
           <t>1. Prompt “Create 3 distinct variations of …” .
 2. Use a reference image and pick a previously generated image.
 3. Edit that image.</t>
         </is>
       </c>
-      <c r="G61" s="2" t="inlineStr">
+      <c r="G62" s="2" t="inlineStr">
         <is>
           <t>Three separate images return, not one combined frame. Reference and prior images work. The edit returns an image preview, not an empty or octet-stream file.</t>
         </is>
       </c>
-      <c r="H61" s="2" t="inlineStr"/>
-      <c r="I61" s="2" t="inlineStr"/>
-    </row>
-    <row r="62" ht="90" customHeight="1">
-      <c r="A62" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="H62" s="2" t="inlineStr"/>
+      <c r="I62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63" ht="90" customHeight="1">
+      <c r="A63" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
         <is>
           <t>1. Customized — Sim behavior Arena changed</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
+      <c r="C63" s="2" t="inlineStr">
         <is>
           <t>Files</t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr">
+      <c r="E63" s="2" t="inlineStr">
         <is>
           <t>Generated images/docs open from file serve route</t>
         </is>
       </c>
-      <c r="F62" s="2" t="inlineStr">
+      <c r="F63" s="2" t="inlineStr">
         <is>
           <t>1. Generate an image and a compiled document.
 2. Open each via the file serve route.
 3. Reuse a chat image in a later run and open that file.</t>
         </is>
       </c>
-      <c r="G62" s="2" t="inlineStr">
+      <c r="G63" s="2" t="inlineStr">
         <is>
           <t>Both open from the file serve route. The reused image is copied onto the run and opens. The path is not a broken or context-query URL.</t>
-        </is>
-      </c>
-      <c r="H62" s="2" t="inlineStr"/>
-      <c r="I62" s="2" t="inlineStr"/>
-    </row>
-    <row r="63" ht="90" customHeight="1">
-      <c r="A63" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>1. Customized — Sim behavior Arena changed</t>
-        </is>
-      </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>Files</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>Org logo upload and display</t>
-        </is>
-      </c>
-      <c r="F63" s="2" t="inlineStr">
-        <is>
-          <t>1. Upload an org logo.
-2. Confirm it displays in the shell/branding surfaces.</t>
-        </is>
-      </c>
-      <c r="G63" s="2" t="inlineStr">
-        <is>
-          <t>Logo uploads and displays correctly.</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr"/>
@@ -2909,18 +2911,18 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Editor file upload can pick chat images</t>
+          <t>Org logo upload and display</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>1. Generate or attach an image in chat.
-2. From the editor file upload, pick an image already in the chat.</t>
+          <t>1. Upload an org logo.
+2. Confirm it displays in the shell/branding surfaces.</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Editor can select images already present in the chat.</t>
+          <t>Logo uploads and displays correctly.</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr"/>
@@ -2932,72 +2934,72 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
+          <t>1. Customized — Sim behavior Arena changed</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Files</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Editor file upload can pick chat images</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>1. Generate or attach an image in chat.
+2. From the editor file upload, pick an image already in the chat.</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Editor can select images already present in the chat.</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr"/>
+      <c r="I65" s="2" t="inlineStr"/>
+    </row>
+    <row r="66" ht="90" customHeight="1">
+      <c r="A66" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
           <t>2. Exclusive — Arena-only</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
         <is>
           <t>Local copilot runtime</t>
         </is>
       </c>
-      <c r="D65" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr">
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
         <is>
           <t>Tool calls, patches, audit history persist across reload</t>
         </is>
       </c>
-      <c r="F65" s="2" t="inlineStr">
+      <c r="F66" s="2" t="inlineStr">
         <is>
           <t>1. On Local, run a turn that performs tool calls / patches.
 2. Reload the page.
 3. Inspect tool calls, patches, and audit history.</t>
         </is>
       </c>
-      <c r="G65" s="2" t="inlineStr">
+      <c r="G66" s="2" t="inlineStr">
         <is>
           <t>Tool calls, patches, and audit history persist across reload.</t>
-        </is>
-      </c>
-      <c r="H65" s="2" t="inlineStr"/>
-      <c r="I65" s="2" t="inlineStr"/>
-    </row>
-    <row r="66" ht="90" customHeight="1">
-      <c r="A66" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>2. Exclusive — Arena-only</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>Local copilot runtime</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="inlineStr">
-        <is>
-          <t>User access and user memory apply to the next turn</t>
-        </is>
-      </c>
-      <c r="F66" s="2" t="inlineStr">
-        <is>
-          <t>1. Configure user access / user memory for Local.
-2. Send a follow-up turn that should use that memory/access.</t>
-        </is>
-      </c>
-      <c r="G66" s="2" t="inlineStr">
-        <is>
-          <t>Next turn respects user access and user memory.</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -3014,67 +3016,67 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
+          <t>Local copilot runtime</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>User access and user memory apply to the next turn</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>1. Configure user access / user memory for Local.
+2. Send a follow-up turn that should use that memory/access.</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>Next turn respects user access and user memory.</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr"/>
+      <c r="I67" s="2" t="inlineStr"/>
+    </row>
+    <row r="68" ht="90" customHeight="1">
+      <c r="A68" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>2. Exclusive — Arena-only</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
           <t>Arena task block</t>
         </is>
       </c>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
         <is>
           <t>Create task / with fields / sub-task / with fields</t>
         </is>
       </c>
-      <c r="F67" s="2" t="inlineStr">
+      <c r="F68" s="2" t="inlineStr">
         <is>
           <t>1. In the Arena block, run create task.
 2. Create task with fields.
 3. Create sub-task and sub-task with fields.</t>
         </is>
       </c>
-      <c r="G67" s="2" t="inlineStr">
+      <c r="G68" s="2" t="inlineStr">
         <is>
           <t>All four create operations succeed and return task data.</t>
-        </is>
-      </c>
-      <c r="H67" s="2" t="inlineStr"/>
-      <c r="I67" s="2" t="inlineStr"/>
-    </row>
-    <row r="68" ht="90" customHeight="1">
-      <c r="A68" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>2. Exclusive — Arena-only</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>Arena task block</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>Add comment / add comment by task number</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="inlineStr">
-        <is>
-          <t>1. Add a comment on a task.
-2. Add a comment by task number.</t>
-        </is>
-      </c>
-      <c r="G68" s="2" t="inlineStr">
-        <is>
-          <t>Both comment operations succeed.</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -3101,135 +3103,135 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
+          <t>Add comment / add comment by task number</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>1. Add a comment on a task.
+2. Add a comment by task number.</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Both comment operations succeed.</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr"/>
+      <c r="I69" s="2" t="inlineStr"/>
+    </row>
+    <row r="70" ht="90" customHeight="1">
+      <c r="A70" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>2. Exclusive — Arena-only</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Arena task block</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
           <t>Fetch searched tasks / search task / simple search</t>
         </is>
       </c>
-      <c r="F69" s="2" t="inlineStr">
+      <c r="F70" s="2" t="inlineStr">
         <is>
           <t>1. Run fetch searched tasks.
 2. Run search task.
 3. Run simple search.</t>
         </is>
       </c>
-      <c r="G69" s="2" t="inlineStr">
+      <c r="G70" s="2" t="inlineStr">
         <is>
           <t>Each search/fetch operation returns matching task data.</t>
         </is>
       </c>
-      <c r="H69" s="2" t="inlineStr"/>
-      <c r="I69" s="2" t="inlineStr"/>
-    </row>
-    <row r="70" ht="90" customHeight="1">
-      <c r="A70" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="B70" s="2" t="inlineStr">
+      <c r="H70" s="2" t="inlineStr"/>
+      <c r="I70" s="2" t="inlineStr"/>
+    </row>
+    <row r="71" ht="90" customHeight="1">
+      <c r="A71" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
         <is>
           <t>2. Exclusive — Arena-only</t>
         </is>
       </c>
-      <c r="C70" s="2" t="inlineStr">
+      <c r="C71" s="2" t="inlineStr">
         <is>
           <t>Arena task block</t>
         </is>
       </c>
-      <c r="D70" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="inlineStr">
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
         <is>
           <t>Save summary / get meetings / get token</t>
         </is>
       </c>
-      <c r="F70" s="2" t="inlineStr">
+      <c r="F71" s="2" t="inlineStr">
         <is>
           <t>1. Run save summary.
 2. Run get meetings.
 3. Run get token.</t>
         </is>
       </c>
-      <c r="G70" s="2" t="inlineStr">
+      <c r="G71" s="2" t="inlineStr">
         <is>
           <t>Each operation succeeds and returns expected payload.</t>
         </is>
       </c>
-      <c r="H70" s="2" t="inlineStr"/>
-      <c r="I70" s="2" t="inlineStr"/>
-    </row>
-    <row r="71" ht="90" customHeight="1">
-      <c r="A71" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="B71" s="2" t="inlineStr">
+      <c r="H71" s="2" t="inlineStr"/>
+      <c r="I71" s="2" t="inlineStr"/>
+    </row>
+    <row r="72" ht="90" customHeight="1">
+      <c r="A72" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
         <is>
           <t>2. Exclusive — Arena-only</t>
         </is>
       </c>
-      <c r="C71" s="2" t="inlineStr">
+      <c r="C72" s="2" t="inlineStr">
         <is>
           <t>Arena task block</t>
         </is>
       </c>
-      <c r="D71" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="E71" s="2" t="inlineStr">
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
         <is>
           <t>Get my tasks / get my overdue tasks</t>
         </is>
       </c>
-      <c r="F71" s="2" t="inlineStr">
+      <c r="F72" s="2" t="inlineStr">
         <is>
           <t>1. Run get my tasks and get my overdue tasks from the builder.
 2. Start the same workflow from a schedule or a webhook and run both operations again.
 3. If Arena auth fails, confirm the block returns an error.</t>
         </is>
       </c>
-      <c r="G71" s="2" t="inlineStr">
+      <c r="G72" s="2" t="inlineStr">
         <is>
           <t>Both operations return the user’s tasks from a manual run and from a schedule or webhook run. A failure is an error, not an empty task list.</t>
-        </is>
-      </c>
-      <c r="H71" s="2" t="inlineStr"/>
-      <c r="I71" s="2" t="inlineStr"/>
-    </row>
-    <row r="72" ht="90" customHeight="1">
-      <c r="A72" s="2" t="n">
-        <v>71</v>
-      </c>
-      <c r="B72" s="2" t="inlineStr">
-        <is>
-          <t>2. Exclusive — Arena-only</t>
-        </is>
-      </c>
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>Arena task block</t>
-        </is>
-      </c>
-      <c r="D72" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="E72" s="2" t="inlineStr">
-        <is>
-          <t>Client and project selectors load Arena data</t>
-        </is>
-      </c>
-      <c r="F72" s="2" t="inlineStr">
-        <is>
-          <t>1. Open the Arena block panel.
-2. Open client and project selectors.</t>
-        </is>
-      </c>
-      <c r="G72" s="2" t="inlineStr">
-        <is>
-          <t>Selectors load real Arena client/project data (not empty stubs / errors).</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
@@ -3246,28 +3248,28 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Arena Development and generated apps</t>
+          <t>Arena task block</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Arena Development: edit an Arena app</t>
+          <t>Client and project selectors load Arena data</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>1. Add Arena Development block.
-2. Edit an existing Arena app.</t>
+          <t>1. Open the Arena block panel.
+2. Open client and project selectors.</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>Edit succeeds and persists for the Arena app.</t>
+          <t>Selectors load real Arena client/project data (not empty stubs / errors).</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr"/>
@@ -3294,57 +3296,57 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
+          <t>Arena Development: edit an Arena app</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>1. Add Arena Development block.
+2. Edit an existing Arena app.</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Edit succeeds and persists for the Arena app.</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr"/>
+      <c r="I74" s="2" t="inlineStr"/>
+    </row>
+    <row r="75" ht="90" customHeight="1">
+      <c r="A75" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>2. Exclusive — Arena-only</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Arena Development and generated apps</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
           <t>Development: generate, edit, deploy to Vercel</t>
         </is>
       </c>
-      <c r="F74" s="2" t="inlineStr">
+      <c r="F75" s="2" t="inlineStr">
         <is>
           <t>1. Generate an app with the Development block.
 2. Edit it.
 3. Deploy to Vercel.</t>
         </is>
       </c>
-      <c r="G74" s="2" t="inlineStr">
+      <c r="G75" s="2" t="inlineStr">
         <is>
           <t>Generate, edit, and Vercel deploy each succeed.</t>
-        </is>
-      </c>
-      <c r="H74" s="2" t="inlineStr"/>
-      <c r="I74" s="2" t="inlineStr"/>
-    </row>
-    <row r="75" ht="90" customHeight="1">
-      <c r="A75" s="2" t="n">
-        <v>74</v>
-      </c>
-      <c r="B75" s="2" t="inlineStr">
-        <is>
-          <t>2. Exclusive — Arena-only</t>
-        </is>
-      </c>
-      <c r="C75" s="2" t="inlineStr">
-        <is>
-          <t>Arena Development and generated apps</t>
-        </is>
-      </c>
-      <c r="D75" s="2" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="E75" s="2" t="inlineStr">
-        <is>
-          <t>Skill share across workspace/org</t>
-        </is>
-      </c>
-      <c r="F75" s="2" t="inlineStr">
-        <is>
-          <t>1. Publish a skill into the catalog.
-2. Use/copy it in another workspace or org.</t>
-        </is>
-      </c>
-      <c r="G75" s="2" t="inlineStr">
-        <is>
-          <t>Published skill is usable from the other workspace/org.</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr"/>
@@ -3361,7 +3363,7 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Exclusive blocks</t>
+          <t>Arena Development and generated apps</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -3371,18 +3373,18 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Bing Ads, Facebook Ads, Google Ads V1</t>
+          <t>Skill share across workspace/org</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>1. Confirm each block appears in the block menu.
-2. Run one NL or GAQL/query op per product.</t>
+          <t>1. Publish a skill into the catalog.
+2. Use/copy it in another workspace or org.</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Blocks appear. One operation per product returns data.</t>
+          <t>Published skill is usable from the other workspace/org.</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -3409,18 +3411,18 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Figma file read or design action</t>
+          <t>Bing Ads, Facebook Ads, Google Ads V1</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>1. Confirm Figma is in the block menu.
-2. Run a file read or design action.</t>
+          <t>1. Confirm each block appears in the block menu.
+2. Run one NL or GAQL/query op per product.</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>Block visible; operation returns data.</t>
+          <t>Blocks appear. One operation per product returns data.</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr"/>
@@ -3447,18 +3449,18 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Image Fusion</t>
+          <t>Figma file read or design action</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>1. Confirm Image Fusion is in the menu.
-2. Fuse two or more images into one output.</t>
+          <t>1. Confirm Figma is in the block menu.
+2. Run a file read or design action.</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Fused image is produced from multiple inputs.</t>
+          <t>Block visible; operation returns data.</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
@@ -3485,18 +3487,18 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>P2 Docs</t>
+          <t>Image Fusion</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>1. Confirm P2 Docs is in the menu.
-2. Run template schema, icons, or team data once.</t>
+          <t>1. Confirm Image Fusion is in the menu.
+2. Fuse two or more images into one output.</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Block visible; chosen operation returns data.</t>
+          <t>Fused image is produced from multiple inputs.</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr"/>
@@ -3523,18 +3525,18 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Semrush and SpyFu</t>
+          <t>P2 Docs</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>1. Confirm both appear in the menu.
-2. Run one SEO query on each.</t>
+          <t>1. Confirm P2 Docs is in the menu.
+2. Run template schema, icons, or team data once.</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>Each returns SEO query data once.</t>
+          <t>Block visible; chosen operation returns data.</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr"/>
@@ -3561,57 +3563,57 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
+          <t>Semrush and SpyFu</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>1. Confirm both appear in the menu.
+2. Run one SEO query on each.</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>Each returns SEO query data once.</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr"/>
+      <c r="I81" s="2" t="inlineStr"/>
+    </row>
+    <row r="82" ht="90" customHeight="1">
+      <c r="A82" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>2. Exclusive — Arena-only</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Exclusive blocks</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
           <t>LinkedIn via Unipile</t>
         </is>
       </c>
-      <c r="F81" s="2" t="inlineStr">
+      <c r="F82" s="2" t="inlineStr">
         <is>
           <t>1. Confirm Unipile/LinkedIn block is available.
 2. Read company or profile.
 3. Exercise hosted auth / reconnect if needed.</t>
         </is>
       </c>
-      <c r="G81" s="2" t="inlineStr">
+      <c r="G82" s="2" t="inlineStr">
         <is>
           <t>Read succeeds. Hosted auth / reconnect works when required.</t>
-        </is>
-      </c>
-      <c r="H81" s="2" t="inlineStr"/>
-      <c r="I81" s="2" t="inlineStr"/>
-    </row>
-    <row r="82" ht="90" customHeight="1">
-      <c r="A82" s="2" t="n">
-        <v>81</v>
-      </c>
-      <c r="B82" s="2" t="inlineStr">
-        <is>
-          <t>2. Exclusive — Arena-only</t>
-        </is>
-      </c>
-      <c r="C82" s="2" t="inlineStr">
-        <is>
-          <t>Exclusive blocks</t>
-        </is>
-      </c>
-      <c r="D82" s="2" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="inlineStr">
-        <is>
-          <t>Chart Generator</t>
-        </is>
-      </c>
-      <c r="F82" s="2" t="inlineStr">
-        <is>
-          <t>1. Confirm Chart Generator is in the menu.
-2. Produce ECharts JSON and render in chat.</t>
-        </is>
-      </c>
-      <c r="G82" s="2" t="inlineStr">
-        <is>
-          <t>Chat renderer draws the chart from the JSON output.</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr"/>
@@ -3638,18 +3640,18 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Skyvern create or get run</t>
+          <t>Chart Generator</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>1. If credentials exist, create or get a Skyvern run.
-2. Otherwise mark N/A with ticket/env note.</t>
+          <t>1. Confirm Chart Generator is in the menu.
+2. Produce ECharts JSON and render in chat.</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>Successful create/get, or explicit N/A with ticket reference when no credential.</t>
+          <t>Chat renderer draws the chart from the JSON output.</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -3676,18 +3678,18 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Airweave successful run</t>
+          <t>Skyvern create or get run</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>1. Confirm Airweave visibility for this product build.
-2. Run once, or N/A with ticket if product does not ship it.</t>
+          <t>1. If credentials exist, create or get a Skyvern run.
+2. Otherwise mark N/A with ticket/env note.</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>One successful run, or N/A with ticket reference.</t>
+          <t>Successful create/get, or explicit N/A with ticket reference when no credential.</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
@@ -3704,28 +3706,28 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Deployed-chat extras</t>
+          <t>Exclusive blocks</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Departments, assistant assets, banners, prompt feedback, golden queries</t>
+          <t>Airweave successful run</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>1. Configure/verify departments, assistant assets, banner messages.
-2. Exercise prompt feedback and workflow golden queries on deployed chat.</t>
+          <t>1. Confirm Airweave visibility for this product build.
+2. Run once, or N/A with ticket if product does not ship it.</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>All Arena-only extras render and function; golden queries work with the extras pack.</t>
+          <t>One successful run, or N/A with ticket reference.</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr"/>
@@ -3752,18 +3754,18 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Thread list in left nav; theme sync with Arena shell</t>
+          <t>Departments, assistant assets, banners, prompt feedback, golden queries</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>1. Open deployed chat left nav thread list.
-2. Compare theme with the Arena shell.</t>
+          <t>1. Configure/verify departments, assistant assets, banner messages.
+2. Exercise prompt feedback and workflow golden queries on deployed chat.</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Thread list works. Theme syncs with the Arena shell.</t>
+          <t>All Arena-only extras render and function; golden queries work with the extras pack.</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
@@ -3780,223 +3782,223 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
+          <t>Deployed-chat extras</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>Thread list in left nav; theme sync with Arena shell</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>1. Open deployed chat left nav thread list.
+2. Compare theme with the Arena shell.</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>Thread list works. Theme syncs with the Arena shell.</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr"/>
+      <c r="I87" s="2" t="inlineStr"/>
+    </row>
+    <row r="88" ht="90" customHeight="1">
+      <c r="A88" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>2. Exclusive — Arena-only</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
           <t>Admin, identity, and ops</t>
         </is>
       </c>
-      <c r="D87" s="2" t="inlineStr">
+      <c r="D88" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E87" s="2" t="inlineStr">
+      <c r="E88" s="2" t="inlineStr">
         <is>
           <t>Arena SSO login, resume, legacy cookie clear</t>
         </is>
       </c>
-      <c r="F87" s="2" t="inlineStr">
+      <c r="F88" s="2" t="inlineStr">
         <is>
           <t>1. Log in via Arena SSO.
 2. Resume a session into Sim.
 3. On a user with an old host-only session cookie, sign out/clear and confirm legacy cookies expire.</t>
         </is>
       </c>
-      <c r="G87" s="2" t="inlineStr">
+      <c r="G88" s="2" t="inlineStr">
         <is>
           <t>Login and resume work. Legacy session cookies are cleared (including __Secure- / Domain variants).</t>
         </is>
       </c>
-      <c r="H87" s="2" t="inlineStr"/>
-      <c r="I87" s="2" t="inlineStr"/>
-    </row>
-    <row r="88" ht="90" customHeight="1">
-      <c r="A88" s="2" t="n">
-        <v>87</v>
-      </c>
-      <c r="B88" s="2" t="inlineStr">
+      <c r="H88" s="2" t="inlineStr"/>
+      <c r="I88" s="2" t="inlineStr"/>
+    </row>
+    <row r="89" ht="90" customHeight="1">
+      <c r="A89" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
         <is>
           <t>2. Exclusive — Arena-only</t>
         </is>
       </c>
-      <c r="C88" s="2" t="inlineStr">
+      <c r="C89" s="2" t="inlineStr">
         <is>
           <t>Admin, identity, and ops</t>
         </is>
       </c>
-      <c r="D88" s="2" t="inlineStr">
+      <c r="D89" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E88" s="2" t="inlineStr">
+      <c r="E89" s="2" t="inlineStr">
         <is>
           <t>Custom OAuth apps at org level</t>
         </is>
       </c>
-      <c r="F88" s="2" t="inlineStr">
+      <c r="F89" s="2" t="inlineStr">
         <is>
           <t>1. Open Settings → Custom OAuth Apps.
 2. Configure an org-level app with allowed workspaces.
 3. Connect from an allowed workspace; try a disallowed one if applicable.</t>
         </is>
       </c>
-      <c r="G88" s="2" t="inlineStr">
+      <c r="G89" s="2" t="inlineStr">
         <is>
           <t>The section shows the apps form, not a blank page. Allowed workspaces can use the app. Restrictions respect org configuration.</t>
         </is>
       </c>
-      <c r="H88" s="2" t="inlineStr"/>
-      <c r="I88" s="2" t="inlineStr"/>
-    </row>
-    <row r="89" ht="90" customHeight="1">
-      <c r="A89" s="2" t="n">
-        <v>88</v>
-      </c>
-      <c r="B89" s="2" t="inlineStr">
+      <c r="H89" s="2" t="inlineStr"/>
+      <c r="I89" s="2" t="inlineStr"/>
+    </row>
+    <row r="90" ht="90" customHeight="1">
+      <c r="A90" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
         <is>
           <t>2. Exclusive — Arena-only</t>
         </is>
       </c>
-      <c r="C89" s="2" t="inlineStr">
+      <c r="C90" s="2" t="inlineStr">
         <is>
           <t>Admin, identity, and ops</t>
         </is>
       </c>
-      <c r="D89" s="2" t="inlineStr">
+      <c r="D90" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E89" s="2" t="inlineStr">
+      <c r="E90" s="2" t="inlineStr">
         <is>
           <t>Agent access requests</t>
         </is>
       </c>
-      <c r="F89" s="2" t="inlineStr">
+      <c r="F90" s="2" t="inlineStr">
         <is>
           <t>1. As a platform-admin email, open Settings → Agent access requests.
 2. Approve one request.
 3. As the requester, open the agents list.</t>
         </is>
       </c>
-      <c r="G89" s="2" t="inlineStr">
+      <c r="G90" s="2" t="inlineStr">
         <is>
           <t>The settings page opens. After approval the requester sees that agent enabled.</t>
         </is>
       </c>
-      <c r="H89" s="2" t="inlineStr"/>
-      <c r="I89" s="2" t="inlineStr"/>
-    </row>
-    <row r="90" ht="90" customHeight="1">
-      <c r="A90" s="2" t="n">
-        <v>89</v>
-      </c>
-      <c r="B90" s="2" t="inlineStr">
+      <c r="H90" s="2" t="inlineStr"/>
+      <c r="I90" s="2" t="inlineStr"/>
+    </row>
+    <row r="91" ht="90" customHeight="1">
+      <c r="A91" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
         <is>
           <t>2. Exclusive — Arena-only</t>
         </is>
       </c>
-      <c r="C90" s="2" t="inlineStr">
+      <c r="C91" s="2" t="inlineStr">
         <is>
           <t>Agents list and video builder</t>
         </is>
       </c>
-      <c r="D90" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="E90" s="2" t="inlineStr">
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
         <is>
           <t>Agents list allow-list and undeploy</t>
         </is>
       </c>
-      <c r="F90" s="2" t="inlineStr">
+      <c r="F91" s="2" t="inlineStr">
         <is>
           <t>1. With an email on an agent allow-list, open global, shared-with-me, and my-agents.
 2. Repeat with an email outside the list.
 3. Undeploy the chat agent and reload each list. Also confirm an inactive chat is absent.</t>
         </is>
       </c>
-      <c r="G90" s="2" t="inlineStr">
+      <c r="G91" s="2" t="inlineStr">
         <is>
           <t>An allowed email sees the agent enabled. An outside email sees it disabled or absent for that tab. Undeploy removes it from all three lists. An inactive chat is not listed.</t>
         </is>
       </c>
-      <c r="H90" s="2" t="inlineStr"/>
-      <c r="I90" s="2" t="inlineStr"/>
-    </row>
-    <row r="91" ht="90" customHeight="1">
-      <c r="A91" s="2" t="n">
-        <v>90</v>
-      </c>
-      <c r="B91" s="2" t="inlineStr">
+      <c r="H91" s="2" t="inlineStr"/>
+      <c r="I91" s="2" t="inlineStr"/>
+    </row>
+    <row r="92" ht="90" customHeight="1">
+      <c r="A92" s="2" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
         <is>
           <t>2. Exclusive — Arena-only</t>
         </is>
       </c>
-      <c r="C91" s="2" t="inlineStr">
+      <c r="C92" s="2" t="inlineStr">
         <is>
           <t>Agents list and video builder</t>
         </is>
       </c>
-      <c r="D91" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="E91" s="2" t="inlineStr">
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
         <is>
           <t>Video builder emailId and Fal usage</t>
         </is>
       </c>
-      <c r="F91" s="2" t="inlineStr">
+      <c r="F92" s="2" t="inlineStr">
         <is>
           <t>1. From the Arena agents list, open the video builder app while signed in.
 2. Open that same agent detail with emailId omitted, and open a different agent with emailId omitted.
 3. Make a Fal call from the video app and open the Arena user’s usage ledger.</t>
         </is>
       </c>
-      <c r="G91" s="2" t="inlineStr">
+      <c r="G92" s="2" t="inlineStr">
         <is>
           <t>The video builder URL has the logged-in email as emailId, replacing any saved email. Omitting emailId still returns the video builder app and rejects every other agent. The Fal call appears on that user’s usage ledger.</t>
-        </is>
-      </c>
-      <c r="H91" s="2" t="inlineStr"/>
-      <c r="I91" s="2" t="inlineStr"/>
-    </row>
-    <row r="92" ht="90" customHeight="1">
-      <c r="A92" s="2" t="n">
-        <v>91</v>
-      </c>
-      <c r="B92" s="2" t="inlineStr">
-        <is>
-          <t>2. Exclusive — Arena-only</t>
-        </is>
-      </c>
-      <c r="C92" s="2" t="inlineStr">
-        <is>
-          <t>Admin, identity, and ops</t>
-        </is>
-      </c>
-      <c r="D92" s="2" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="E92" s="2" t="inlineStr">
-        <is>
-          <t>Help and support issue filed and stored</t>
-        </is>
-      </c>
-      <c r="F92" s="2" t="inlineStr">
-        <is>
-          <t>1. File a help/support issue via the Arena help path.
-2. Confirm it is stored (DB / admin view).</t>
-        </is>
-      </c>
-      <c r="G92" s="2" t="inlineStr">
-        <is>
-          <t>Issue is accepted and stored.</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr"/>
@@ -4023,18 +4025,18 @@
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>App banner route and workspace embed page</t>
+          <t>Help and support issue filed and stored</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>1. Open the app banner route inside the host frame.
-2. Open the workspace embed page inside the host frame.</t>
+          <t>1. File a help/support issue via the Arena help path.
+2. Confirm it is stored (DB / admin view).</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>Both render correctly inside the host frame.</t>
+          <t>Issue is accepted and stored.</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr"/>
@@ -4061,18 +4063,18 @@
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>Default workflows import and deploy for new user</t>
+          <t>App banner route and workspace embed page</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>1. Provision or use a new user.
-2. Confirm default workflows import and can deploy.</t>
+          <t>1. Open the app banner route inside the host frame.
+2. Open the workspace embed page inside the host frame.</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>Default workflows import and deploy for the new user.</t>
+          <t>Both render correctly inside the host frame.</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr"/>
@@ -4099,18 +4101,18 @@
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>User knowledge base populate attaches to user</t>
+          <t>Default workflows import and deploy for new user</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>1. Trigger user knowledge base populate.
-2. Confirm attachment to the user.</t>
+          <t>1. Provision or use a new user.
+2. Confirm default workflows import and can deploy.</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>KB populate attaches to the user and is usable afterward.</t>
+          <t>Default workflows import and deploy for the new user.</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr"/>
@@ -4137,10 +4139,48 @@
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
+          <t>User knowledge base populate attaches to user</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>1. Trigger user knowledge base populate.
+2. Confirm attachment to the user.</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>KB populate attaches to the user and is usable afterward.</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr"/>
+      <c r="I96" s="2" t="inlineStr"/>
+    </row>
+    <row r="97" ht="90" customHeight="1">
+      <c r="A97" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>2. Exclusive — Arena-only</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Admin, identity, and ops</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
           <t>Arena general settings (timezone and events)</t>
         </is>
       </c>
-      <c r="F96" s="2" t="inlineStr">
+      <c r="F97" s="2" t="inlineStr">
         <is>
           <t>1. Open /workspace/arena-general-settings (no workspace id required).
 2. Save timezone and events.
@@ -4148,47 +4188,9 @@
 4. Spot-check workspace /settings/general still works.</t>
         </is>
       </c>
-      <c r="G96" s="2" t="inlineStr">
+      <c r="G97" s="2" t="inlineStr">
         <is>
           <t>Page opens without a workspace id. Timezone/events save and apply to chat and copilot. Workspace general settings unchanged.</t>
-        </is>
-      </c>
-      <c r="H96" s="2" t="inlineStr"/>
-      <c r="I96" s="2" t="inlineStr"/>
-    </row>
-    <row r="97" ht="90" customHeight="1">
-      <c r="A97" s="2" t="n">
-        <v>96</v>
-      </c>
-      <c r="B97" s="2" t="inlineStr">
-        <is>
-          <t>2. Exclusive — Arena-only</t>
-        </is>
-      </c>
-      <c r="C97" s="2" t="inlineStr">
-        <is>
-          <t>Billing package (Arena-only)</t>
-        </is>
-      </c>
-      <c r="D97" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="E97" s="2" t="inlineStr">
-        <is>
-          <t>Starter provisioned for a new client org</t>
-        </is>
-      </c>
-      <c r="F97" s="2" t="inlineStr">
-        <is>
-          <t>1. Provision a new client org through the Arena path.
-2. Inspect subscription / usage limit.</t>
-        </is>
-      </c>
-      <c r="G97" s="2" t="inlineStr">
-        <is>
-          <t>Starter is provisioned with expected usage limit / metadata.</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr"/>
@@ -4215,57 +4217,57 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
+          <t>Starter provisioned for a new client org</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>1. Provision a new client org through the Arena path.
+2. Inspect subscription / usage limit.</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>Starter is provisioned with expected usage limit / metadata.</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr"/>
+      <c r="I98" s="2" t="inlineStr"/>
+    </row>
+    <row r="99" ht="90" customHeight="1">
+      <c r="A99" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>2. Exclusive — Arena-only</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>Billing package (Arena-only)</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
           <t>Pro and Max checkout (team_1950 / team_6500)</t>
         </is>
       </c>
-      <c r="F98" s="2" t="inlineStr">
+      <c r="F99" s="2" t="inlineStr">
         <is>
           <t>1. As org admin, open upgrade.
 2. Start Pro (team_1950) and/or Max (team_6500) checkout.
 3. Confirm Starter Stripe id is not used for paid checkout.</t>
         </is>
       </c>
-      <c r="G98" s="2" t="inlineStr">
+      <c r="G99" s="2" t="inlineStr">
         <is>
           <t>Catalog shows Pro/Max flat org pricing. Checkout ignores Starter Stripe id. Paid checkout can proceed from active Starter.</t>
-        </is>
-      </c>
-      <c r="H98" s="2" t="inlineStr"/>
-      <c r="I98" s="2" t="inlineStr"/>
-    </row>
-    <row r="99" ht="90" customHeight="1">
-      <c r="A99" s="2" t="n">
-        <v>98</v>
-      </c>
-      <c r="B99" s="2" t="inlineStr">
-        <is>
-          <t>2. Exclusive — Arena-only</t>
-        </is>
-      </c>
-      <c r="C99" s="2" t="inlineStr">
-        <is>
-          <t>Billing package (Arena-only)</t>
-        </is>
-      </c>
-      <c r="D99" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="E99" s="2" t="inlineStr">
-        <is>
-          <t>Org-admin upgrade comparison overlay</t>
-        </is>
-      </c>
-      <c r="F99" s="2" t="inlineStr">
-        <is>
-          <t>1. As org admin, open the upgrade comparison overlay.
-2. Review Starter / Max / Enterprise columns (Pro hidden from comparison table).</t>
-        </is>
-      </c>
-      <c r="G99" s="2" t="inlineStr">
-        <is>
-          <t>Overlay shows Arena comparison with flat org pricing copy. Pro is not a comparison column.</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr"/>
@@ -4292,18 +4294,18 @@
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Seat reconcile does not fight flat org pricing</t>
+          <t>Org-admin upgrade comparison overlay</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>1. With an Arena flat org plan, adjust seats / membership.
-2. Observe seat reconcile / pricing behaviour.</t>
+          <t>1. As org admin, open the upgrade comparison overlay.
+2. Review Starter / Max / Enterprise columns (Pro hidden from comparison table).</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>Seat reconcile does not multiply or fight flat org pricing.</t>
+          <t>Overlay shows Arena comparison with flat org pricing copy. Pro is not a comparison column.</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr"/>
@@ -4330,18 +4332,18 @@
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>Usage limit blocks when exhausted; allows when not</t>
+          <t>Seat reconcile does not fight flat org pricing</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>1. With credits remaining, run a billable action.
-2. Exhaust credits (or use a test org at limit) and retry.</t>
+          <t>1. With an Arena flat org plan, adjust seats / membership.
+2. Observe seat reconcile / pricing behaviour.</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>Run allowed under limit. Run blocked when credits are exhausted.</t>
+          <t>Seat reconcile does not multiply or fight flat org pricing.</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr"/>
@@ -4368,18 +4370,18 @@
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>Paying supersedes Starter; client-org Starter still provisions</t>
+          <t>Usage limit blocks when exhausted; allows when not</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>1. Confirm a new client org still gets Starter.
-2. Complete paid checkout and verify Starter is superseded.</t>
+          <t>1. With credits remaining, run a billable action.
+2. Exhaust credits (or use a test org at limit) and retry.</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>Starter provisioning still runs for client orgs. Paying supersedes Starter.</t>
+          <t>Run allowed under limit. Run blocked when credits are exhausted.</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr"/>
@@ -4391,12 +4393,12 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>3. Other Sim features — stock regression</t>
+          <t>2. Exclusive — Arena-only</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>Builder core</t>
+          <t>Billing package (Arena-only)</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
@@ -4406,18 +4408,18 @@
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>Create, rename, duplicate, delete; undo/redo</t>
+          <t>Paying supersedes Starter; client-org Starter still provisions</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>1. Create a workflow; rename; duplicate; delete.
-2. Exercise undo and redo on canvas edits.</t>
+          <t>1. Confirm a new client org still gets Starter.
+2. Complete paid checkout and verify Starter is superseded.</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>CRUD works. Undo/redo restores prior canvas state.</t>
+          <t>Starter provisioning still runs for client orgs. Paying supersedes Starter.</t>
         </is>
       </c>
       <c r="H103" s="2" t="inlineStr"/>
@@ -4444,96 +4446,96 @@
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
+          <t>Create, rename, duplicate, delete; undo/redo</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>1. Create a workflow; rename; duplicate; delete.
+2. Exercise undo and redo on canvas edits.</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>CRUD works. Undo/redo restores prior canvas state.</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr"/>
+      <c r="I104" s="2" t="inlineStr"/>
+    </row>
+    <row r="105" ht="90" customHeight="1">
+      <c r="A105" s="2" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>3. Other Sim features — stock regression</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>Builder core</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
           <t>Drag blocks, connect edges, editor panel, variables</t>
         </is>
       </c>
-      <c r="F104" s="2" t="inlineStr">
+      <c r="F105" s="2" t="inlineStr">
         <is>
           <t>1. Drag blocks onto the canvas and connect edges.
 2. Open the editor panel.
 3. Use a &lt;Block.output&gt; variable reference.</t>
         </is>
       </c>
-      <c r="G104" s="2" t="inlineStr">
+      <c r="G105" s="2" t="inlineStr">
         <is>
           <t>Blocks connect. Panel opens. Variables resolve.</t>
         </is>
       </c>
-      <c r="H104" s="2" t="inlineStr"/>
-      <c r="I104" s="2" t="inlineStr"/>
-    </row>
-    <row r="105" ht="90" customHeight="1">
-      <c r="A105" s="2" t="n">
-        <v>104</v>
-      </c>
-      <c r="B105" s="2" t="inlineStr">
+      <c r="H105" s="2" t="inlineStr"/>
+      <c r="I105" s="2" t="inlineStr"/>
+    </row>
+    <row r="106" ht="90" customHeight="1">
+      <c r="A106" s="2" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
         <is>
           <t>3. Other Sim features — stock regression</t>
         </is>
       </c>
-      <c r="C105" s="2" t="inlineStr">
+      <c r="C106" s="2" t="inlineStr">
         <is>
           <t>Builder core</t>
         </is>
       </c>
-      <c r="D105" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="E105" s="2" t="inlineStr">
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
         <is>
           <t>Manual run, stop, console; logs page</t>
         </is>
       </c>
-      <c r="F105" s="2" t="inlineStr">
+      <c r="F106" s="2" t="inlineStr">
         <is>
           <t>1. Manual run a workflow; stop mid-run if possible.
 2. Read the console.
 3. Open the Logs page for the same run.</t>
         </is>
       </c>
-      <c r="G105" s="2" t="inlineStr">
+      <c r="G106" s="2" t="inlineStr">
         <is>
           <t>Run/stop/console work. Logs page shows the same run.</t>
-        </is>
-      </c>
-      <c r="H105" s="2" t="inlineStr"/>
-      <c r="I105" s="2" t="inlineStr"/>
-    </row>
-    <row r="106" ht="90" customHeight="1">
-      <c r="A106" s="2" t="n">
-        <v>105</v>
-      </c>
-      <c r="B106" s="2" t="inlineStr">
-        <is>
-          <t>3. Other Sim features — stock regression</t>
-        </is>
-      </c>
-      <c r="C106" s="2" t="inlineStr">
-        <is>
-          <t>Builder core</t>
-        </is>
-      </c>
-      <c r="D106" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="E106" s="2" t="inlineStr">
-        <is>
-          <t>Save/reload; realtime second user</t>
-        </is>
-      </c>
-      <c r="F106" s="2" t="inlineStr">
-        <is>
-          <t>1. Save and reload the workflow.
-2. Have a second user open the same workflow and make an edit.</t>
-        </is>
-      </c>
-      <c r="G106" s="2" t="inlineStr">
-        <is>
-          <t>State persists after reload. Second user sees realtime updates.</t>
         </is>
       </c>
       <c r="H106" s="2" t="inlineStr"/>
@@ -4560,18 +4562,18 @@
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>Deploy; API trigger and chat trigger</t>
+          <t>Save/reload; realtime second user</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>1. Deploy the workflow.
-2. Fire an API trigger and a chat trigger.</t>
+          <t>1. Save and reload the workflow.
+2. Have a second user open the same workflow and make an edit.</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>Each trigger starts a run successfully.</t>
+          <t>State persists after reload. Second user sees realtime updates.</t>
         </is>
       </c>
       <c r="H107" s="2" t="inlineStr"/>
@@ -4598,18 +4600,18 @@
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>Schedule trigger and webhook trigger</t>
+          <t>Deploy; API trigger and chat trigger</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>1. Configure a schedule; wait for one fire (or advance in test env).
-2. Send one signed webhook request.</t>
+          <t>1. Deploy the workflow.
+2. Fire an API trigger and a chat trigger.</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>Schedule fires once. Webhook accepts the signed request and starts a run.</t>
+          <t>Each trigger starts a run successfully.</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr"/>
@@ -4636,18 +4638,18 @@
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>Response body; Condition and Router branches</t>
+          <t>Schedule trigger and webhook trigger</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>1. Configure a Response block body and run.
-2. Configure Condition and Router; take each branch once.</t>
+          <t>1. Configure a schedule; wait for one fire (or advance in test env).
+2. Send one signed webhook request.</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>Response returns configured body. Condition and Router take the correct branch.</t>
+          <t>Schedule fires once. Webhook accepts the signed request and starts a run.</t>
         </is>
       </c>
       <c r="H109" s="2" t="inlineStr"/>
@@ -4674,56 +4676,57 @@
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
+          <t>Response body; Condition and Router branches</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>1. Configure a Response block body and run.
+2. Configure Condition and Router; take each branch once.</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>Response returns configured body. Condition and Router take the correct branch.</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr"/>
+      <c r="I110" s="2" t="inlineStr"/>
+    </row>
+    <row r="111" ht="90" customHeight="1">
+      <c r="A111" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>3. Other Sim features — stock regression</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>Builder core</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
           <t>Loop and parallel small inner graph</t>
         </is>
       </c>
-      <c r="F110" s="2" t="inlineStr">
+      <c r="F111" s="2" t="inlineStr">
         <is>
           <t>1. Run a small loop inner graph.
 2. Run a small parallel inner graph.
 3. (Nested Arena case already covered in section 1.)</t>
         </is>
       </c>
-      <c r="G110" s="2" t="inlineStr">
+      <c r="G111" s="2" t="inlineStr">
         <is>
           <t>Loop and parallel each run the inner graph correctly.</t>
-        </is>
-      </c>
-      <c r="H110" s="2" t="inlineStr"/>
-      <c r="I110" s="2" t="inlineStr"/>
-    </row>
-    <row r="111" ht="90" customHeight="1">
-      <c r="A111" s="2" t="n">
-        <v>110</v>
-      </c>
-      <c r="B111" s="2" t="inlineStr">
-        <is>
-          <t>3. Other Sim features — stock regression</t>
-        </is>
-      </c>
-      <c r="C111" s="2" t="inlineStr">
-        <is>
-          <t>Workspace surfaces</t>
-        </is>
-      </c>
-      <c r="D111" s="2" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="E111" s="2" t="inlineStr">
-        <is>
-          <t>Home, workflow list, sidebar navigation</t>
-        </is>
-      </c>
-      <c r="F111" s="2" t="inlineStr">
-        <is>
-          <t>1. Open home, workflow list, and navigate the sidebar.</t>
-        </is>
-      </c>
-      <c r="G111" s="2" t="inlineStr">
-        <is>
-          <t>All surfaces load and navigate without errors.</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr"/>
@@ -4750,56 +4753,56 @@
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
+          <t>Home, workflow list, sidebar navigation</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>1. Open home, workflow list, and navigate the sidebar.</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>All surfaces load and navigate without errors.</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr"/>
+      <c r="I112" s="2" t="inlineStr"/>
+    </row>
+    <row r="113" ht="90" customHeight="1">
+      <c r="A113" s="2" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>3. Other Sim features — stock regression</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>Workspace surfaces</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
           <t>Knowledge: create base, upload, retrieve from Agent</t>
         </is>
       </c>
-      <c r="F112" s="2" t="inlineStr">
+      <c r="F113" s="2" t="inlineStr">
         <is>
           <t>1. Create a knowledge base; upload a document.
 2. Retrieve it from an Agent block.
 3. Run a search that hits and a search that matches nothing.</t>
         </is>
       </c>
-      <c r="G112" s="2" t="inlineStr">
+      <c r="G113" s="2" t="inlineStr">
         <is>
           <t>Upload succeeds. Agent retrieval returns the document content/citations. A hit includes rank. An empty search returns an empty result the Agent can consume, with no crash on a missing rank.</t>
-        </is>
-      </c>
-      <c r="H112" s="2" t="inlineStr"/>
-      <c r="I112" s="2" t="inlineStr"/>
-    </row>
-    <row r="113" ht="90" customHeight="1">
-      <c r="A113" s="2" t="n">
-        <v>112</v>
-      </c>
-      <c r="B113" s="2" t="inlineStr">
-        <is>
-          <t>3. Other Sim features — stock regression</t>
-        </is>
-      </c>
-      <c r="C113" s="2" t="inlineStr">
-        <is>
-          <t>Workspace surfaces</t>
-        </is>
-      </c>
-      <c r="D113" s="2" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="E113" s="2" t="inlineStr">
-        <is>
-          <t>Tables: create, add row, filter</t>
-        </is>
-      </c>
-      <c r="F113" s="2" t="inlineStr">
-        <is>
-          <t>1. Create a table; add a row; apply a filter.</t>
-        </is>
-      </c>
-      <c r="G113" s="2" t="inlineStr">
-        <is>
-          <t>Row appears and filter returns the expected subset.</t>
         </is>
       </c>
       <c r="H113" s="2" t="inlineStr"/>
@@ -4826,18 +4829,17 @@
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
-          <t>Files: upload, preview PDF/image, delete</t>
+          <t>Tables: create, add row, filter</t>
         </is>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>1. Upload a PDF and an image.
-2. Preview each; delete one.</t>
+          <t>1. Create a table; add a row; apply a filter.</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
-          <t>Upload/preview/delete succeed for PDF and image.</t>
+          <t>Row appears and filter returns the expected subset.</t>
         </is>
       </c>
       <c r="H114" s="2" t="inlineStr"/>
@@ -4864,18 +4866,18 @@
       </c>
       <c r="E115" s="2" t="inlineStr">
         <is>
-          <t>Skills: create and attach to agent</t>
+          <t>Files: upload, preview PDF/image, delete</t>
         </is>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>1. Create a skill.
-2. Attach it to an agent and run once.</t>
+          <t>1. Upload a PDF and an image.
+2. Preview each; delete one.</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>Skill attaches and is used by the agent run.</t>
+          <t>Upload/preview/delete succeed for PDF and image.</t>
         </is>
       </c>
       <c r="H115" s="2" t="inlineStr"/>
@@ -4902,17 +4904,18 @@
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>Logs, tests, dashboards, changelog pages load</t>
+          <t>Skills: create and attach to agent</t>
         </is>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>1. Open logs, tests, dashboards, and changelog pages.</t>
+          <t>1. Create a skill.
+2. Attach it to an agent and run once.</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>Each page loads without error.</t>
+          <t>Skill attaches and is used by the agent run.</t>
         </is>
       </c>
       <c r="H116" s="2" t="inlineStr"/>
@@ -4939,18 +4942,17 @@
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t>Integrations catalog and connected credential</t>
+          <t>Logs, tests, dashboards, changelog pages load</t>
         </is>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>1. Open the integrations catalog.
-2. Open a connected credential detail.</t>
+          <t>1. Open logs, tests, dashboards, and changelog pages.</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>Catalog and credential detail both open.</t>
+          <t>Each page loads without error.</t>
         </is>
       </c>
       <c r="H117" s="2" t="inlineStr"/>
@@ -4977,18 +4979,18 @@
       </c>
       <c r="E118" s="2" t="inlineStr">
         <is>
-          <t>Recently deleted: restore one workflow</t>
+          <t>Integrations catalog and connected credential</t>
         </is>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>1. Delete a workflow.
-2. Restore it from Recently deleted.</t>
+          <t>1. Open the integrations catalog.
+2. Open a connected credential detail.</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>Workflow restores and opens.</t>
+          <t>Catalog and credential detail both open.</t>
         </is>
       </c>
       <c r="H118" s="2" t="inlineStr"/>
@@ -5005,7 +5007,7 @@
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Workspace surfaces</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
@@ -5015,17 +5017,18 @@
       </c>
       <c r="E119" s="2" t="inlineStr">
         <is>
-          <t>Account, teammates, org members, secrets, credential groups</t>
+          <t>Recently deleted: restore one workflow</t>
         </is>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>1. Open each settings page and perform a trivial save/view.</t>
+          <t>1. Delete a workflow.
+2. Restore it from Recently deleted.</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>Each page loads; trivial actions succeed.</t>
+          <t>Workflow restores and opens.</t>
         </is>
       </c>
       <c r="H119" s="2" t="inlineStr"/>
@@ -5052,57 +5055,56 @@
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
+          <t>Account, teammates, org members, secrets, credential groups</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>1. Open each settings page and perform a trivial save/view.</t>
+        </is>
+      </c>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>Each page loads; trivial actions succeed.</t>
+        </is>
+      </c>
+      <c r="H120" s="2" t="inlineStr"/>
+      <c r="I120" s="2" t="inlineStr"/>
+    </row>
+    <row r="121" ht="90" customHeight="1">
+      <c r="A121" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>3. Other Sim features — stock regression</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
           <t>Arena API keys: create, use on API trigger, revoke</t>
         </is>
       </c>
-      <c r="F120" s="2" t="inlineStr">
+      <c r="F121" s="2" t="inlineStr">
         <is>
           <t>1. Create an Arena API key.
 2. Use it on an API trigger.
 3. Revoke it and confirm rejection.</t>
         </is>
       </c>
-      <c r="G120" s="2" t="inlineStr">
+      <c r="G121" s="2" t="inlineStr">
         <is>
           <t>Create/use succeed. After revoke, the key is rejected.</t>
-        </is>
-      </c>
-      <c r="H120" s="2" t="inlineStr"/>
-      <c r="I120" s="2" t="inlineStr"/>
-    </row>
-    <row r="121" ht="90" customHeight="1">
-      <c r="A121" s="2" t="n">
-        <v>120</v>
-      </c>
-      <c r="B121" s="2" t="inlineStr">
-        <is>
-          <t>3. Other Sim features — stock regression</t>
-        </is>
-      </c>
-      <c r="C121" s="2" t="inlineStr">
-        <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="D121" s="2" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="E121" s="2" t="inlineStr">
-        <is>
-          <t>Custom tools, MCP tools, MCP servers, sandboxes</t>
-        </is>
-      </c>
-      <c r="F121" s="2" t="inlineStr">
-        <is>
-          <t>1. Open each settings surface.
-2. Spot-check one create/connect action if credentials allow.</t>
-        </is>
-      </c>
-      <c r="G121" s="2" t="inlineStr">
-        <is>
-          <t>Surfaces load; spot-check action succeeds or is N/A with reason.</t>
         </is>
       </c>
       <c r="H121" s="2" t="inlineStr"/>
@@ -5129,18 +5131,18 @@
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>Permission groups and audit logs (enterprise)</t>
+          <t>Custom tools, MCP tools, MCP servers, sandboxes</t>
         </is>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>1. If the org has enterprise, open permission groups and audit logs.
-2. Otherwise mark N/A.</t>
+          <t>1. Open each settings surface.
+2. Spot-check one create/connect action if credentials allow.</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
-          <t>Pages load for enterprise orgs; N/A otherwise.</t>
+          <t>Surfaces load; spot-check action succeeds or is N/A with reason.</t>
         </is>
       </c>
       <c r="H122" s="2" t="inlineStr"/>
@@ -5167,18 +5169,18 @@
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
-          <t>Subscription page matches Arena plan</t>
+          <t>Permission groups and audit logs (enterprise)</t>
         </is>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>1. Open the subscription page.
-2. Compare to the Arena plan verified in section 2 billing.</t>
+          <t>1. If the org has enterprise, open permission groups and audit logs.
+2. Otherwise mark N/A.</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
-          <t>Subscription page matches the Arena plan (Starter/Pro/Max).</t>
+          <t>Pages load for enterprise orgs; N/A otherwise.</t>
         </is>
       </c>
       <c r="H123" s="2" t="inlineStr"/>
@@ -5195,28 +5197,28 @@
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>Agent and model path</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>Agent block calls allowed model and returns text</t>
+          <t>Subscription page matches Arena plan</t>
         </is>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>1. Configure an Agent block with one allowed model.
-2. Run and read the text output.</t>
+          <t>1. Open the subscription page.
+2. Compare to the Arena plan verified in section 2 billing.</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
         <is>
-          <t>Agent returns text from the allowed model.</t>
+          <t>Subscription page matches the Arena plan (Starter/Pro/Max).</t>
         </is>
       </c>
       <c r="H124" s="2" t="inlineStr"/>
@@ -5243,18 +5245,18 @@
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>Tools the agent calls show in the trace</t>
+          <t>Agent block calls allowed model and returns text</t>
         </is>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>1. Run an Agent that calls at least one tool.
-2. Inspect the run trace.</t>
+          <t>1. Configure an Agent block with one allowed model.
+2. Run and read the text output.</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>Tool calls appear in the trace.</t>
+          <t>Agent returns text from the allowed model.</t>
         </is>
       </c>
       <c r="H125" s="2" t="inlineStr"/>
@@ -5281,18 +5283,18 @@
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>Memory survives a second run in the same thread</t>
+          <t>Tools the agent calls show in the trace</t>
         </is>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>1. Run an Agent with memory in a thread.
-2. Run a second turn in the same thread that depends on memory.</t>
+          <t>1. Run an Agent that calls at least one tool.
+2. Inspect the run trace.</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>Second run uses memory from the first.</t>
+          <t>Tool calls appear in the trace.</t>
         </is>
       </c>
       <c r="H126" s="2" t="inlineStr"/>
@@ -5309,28 +5311,28 @@
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>Representative stock integrations</t>
+          <t>Agent and model path</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
-          <t>Google: Calendar, Sheets, Docs (Gmail/Drive covered in §1)</t>
+          <t>Memory survives a second run in the same thread</t>
         </is>
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>1. If credentials exist, run one read/write each for Calendar, Sheets, Docs.
-2. Skip Gmail/Drive here if already passed in section 1 Extended; note in Notes.</t>
+          <t>1. Run an Agent with memory in a thread.
+2. Run a second turn in the same thread that depends on memory.</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>Each tested Google service succeeds once, or N/A with credential note. Gmail/Drive may be N/A-if-covered-in-§1.</t>
+          <t>Second run uses memory from the first.</t>
         </is>
       </c>
       <c r="H127" s="2" t="inlineStr"/>
@@ -5357,17 +5359,18 @@
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>Microsoft: Outlook, Teams, OneDrive</t>
+          <t>Google: Calendar, Sheets, Docs (Gmail/Drive covered in §1)</t>
         </is>
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>1. With a test account, run one read or write each.</t>
+          <t>1. If credentials exist, run one read/write each for Calendar, Sheets, Docs.
+2. Skip Gmail/Drive here if already passed in section 1 Extended; note in Notes.</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>Each succeeds once, or N/A if no credential.</t>
+          <t>Each tested Google service succeeds once, or N/A with credential note. Gmail/Drive may be N/A-if-covered-in-§1.</t>
         </is>
       </c>
       <c r="H128" s="2" t="inlineStr"/>
@@ -5394,12 +5397,12 @@
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>Atlassian: Jira, Confluence</t>
+          <t>Microsoft: Outlook, Teams, OneDrive</t>
         </is>
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>1. Run one Jira and one Confluence happy path.</t>
+          <t>1. With a test account, run one read or write each.</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -5431,13 +5434,12 @@
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>Dev: GitHub, Linear (or Jira if Linear unavailable)</t>
+          <t>Atlassian: Jira, Confluence</t>
         </is>
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>1. Run one GitHub action.
-2. Run one Linear or Jira action.</t>
+          <t>1. Run one Jira and one Confluence happy path.</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -5469,18 +5471,18 @@
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>Comms: Discord and Microsoft Teams (Slack covered in §1)</t>
+          <t>Dev: GitHub, Linear (or Jira if Linear unavailable)</t>
         </is>
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>1. Run Discord and Teams stock ops.
-2. Mark Slack N/A if already covered by section 1 Extended Slack.</t>
+          <t>1. Run one GitHub action.
+2. Run one Linear or Jira action.</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>Discord/Teams succeed once, or N/A. Slack noted as covered in §1 when applicable.</t>
+          <t>Each succeeds once, or N/A if no credential.</t>
         </is>
       </c>
       <c r="H131" s="2" t="inlineStr"/>
@@ -5507,18 +5509,18 @@
       </c>
       <c r="E132" s="2" t="inlineStr">
         <is>
-          <t>CRM: Salesforce stock read (HubSpot covered in §1)</t>
+          <t>Comms: Discord and Microsoft Teams (Slack covered in §1)</t>
         </is>
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>1. Run a Salesforce stock read if credentialed.
-2. Mark HubSpot N/A if already covered in section 1.</t>
+          <t>1. Run Discord and Teams stock ops.
+2. Mark Slack N/A if already covered by section 1 Extended Slack.</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
-          <t>Salesforce succeeds once, or N/A. HubSpot noted as covered in §1 when applicable.</t>
+          <t>Discord/Teams succeed once, or N/A. Slack noted as covered in §1 when applicable.</t>
         </is>
       </c>
       <c r="H132" s="2" t="inlineStr"/>
@@ -5545,18 +5547,18 @@
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>Data: Airtable or Notion; Postgres or built-in table</t>
+          <t>CRM: Salesforce stock read (HubSpot covered in §1)</t>
         </is>
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>1. Run one Airtable or Notion op.
-2. Run one Postgres or built-in table op.</t>
+          <t>1. Run a Salesforce stock read if credentialed.
+2. Mark HubSpot N/A if already covered in section 1.</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
         <is>
-          <t>Each chosen path succeeds once, or N/A if no credential.</t>
+          <t>Salesforce succeeds once, or N/A. HubSpot noted as covered in §1 when applicable.</t>
         </is>
       </c>
       <c r="H133" s="2" t="inlineStr"/>
@@ -5583,17 +5585,18 @@
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>AI utilities: Search, Function, API block, Evaluator</t>
+          <t>Data: Airtable or Notion; Postgres or built-in table</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>1. Run one happy path each for Search, Function, API block, Evaluator.</t>
+          <t>1. Run one Airtable or Notion op.
+2. Run one Postgres or built-in table op.</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>All four succeed once.</t>
+          <t>Each chosen path succeeds once, or N/A if no credential.</t>
         </is>
       </c>
       <c r="H134" s="2" t="inlineStr"/>
@@ -5610,28 +5613,27 @@
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>Auth and tenancy</t>
+          <t>Representative stock integrations</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>Email sign-in and sign-out; invite and accept</t>
+          <t>AI utilities: Search, Function, API block, Evaluator</t>
         </is>
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>1. Sign in with email; sign out.
-2. Invite a member and accept the invite.</t>
+          <t>1. Run one happy path each for Search, Function, API block, Evaluator.</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
-          <t>Sign-in/out work. Invite accept grants membership.</t>
+          <t>All four succeed once.</t>
         </is>
       </c>
       <c r="H135" s="2" t="inlineStr"/>
@@ -5658,17 +5660,18 @@
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>Member cannot open another org’s workspace</t>
+          <t>Email sign-in and sign-out; invite and accept</t>
         </is>
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>1. As a member of org A, attempt to open org B’s workspace URL.</t>
+          <t>1. Sign in with email; sign out.
+2. Invite a member and accept the invite.</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
-          <t>Access is denied; workspace from another org is not opened.</t>
+          <t>Sign-in/out work. Invite accept grants membership.</t>
         </is>
       </c>
       <c r="H136" s="2" t="inlineStr"/>
@@ -5695,18 +5698,17 @@
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>Archived workspace is not selectable</t>
+          <t>Member cannot open another org’s workspace</t>
         </is>
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>1. Archive a workspace (or use a known archived one).
-2. Try to select it from the workspace picker.</t>
+          <t>1. As a member of org A, attempt to open org B’s workspace URL.</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>Archived workspace is not selectable.</t>
+          <t>Access is denied; workspace from another org is not opened.</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr"/>
@@ -5733,27 +5735,65 @@
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
+          <t>Archived workspace is not selectable</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>1. Archive a workspace (or use a known archived one).
+2. Try to select it from the workspace picker.</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>Archived workspace is not selectable.</t>
+        </is>
+      </c>
+      <c r="H138" s="2" t="inlineStr"/>
+      <c r="I138" s="2" t="inlineStr"/>
+    </row>
+    <row r="139" ht="90" customHeight="1">
+      <c r="A139" s="2" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>3. Other Sim features — stock regression</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>Auth and tenancy</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
           <t>API key from another workspace is rejected</t>
         </is>
       </c>
-      <c r="F138" s="2" t="inlineStr">
+      <c r="F139" s="2" t="inlineStr">
         <is>
           <t>1. Take an API key from workspace A.
 2. Call a protected API scoped to workspace B.</t>
         </is>
       </c>
-      <c r="G138" s="2" t="inlineStr">
+      <c r="G139" s="2" t="inlineStr">
         <is>
           <t>Request is rejected (unauthorized / wrong workspace).</t>
         </is>
       </c>
-      <c r="H138" s="2" t="inlineStr"/>
-      <c r="I138" s="2" t="inlineStr"/>
+      <c r="H139" s="2" t="inlineStr"/>
+      <c r="I139" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I138"/>
+  <autoFilter ref="A1:I139"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H138" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid result" error="Choose Pass, Fail, or N/A" type="list">
+    <dataValidation sqref="H2:H139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid result" error="Choose Pass, Fail, or N/A" type="list">
       <formula1>"Pass,Fail,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5929,7 +5969,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Kept rows: 137 (P0=77, P1=39, P2=21)</t>
+          <t>Kept rows: 138 (P0=78, P1=39, P2=21)</t>
         </is>
       </c>
     </row>

</xml_diff>